<commit_message>
Correct measure range in a repeat-sign question
Narrow the range from measures 1-256 to 1-200.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/msu-bench.xlsx
+++ b/msu-bench.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>In measures 1–256, is there a repeat sign?</t>
+          <t>In measures 1–200, is there a repeat sign?</t>
         </is>
       </c>
       <c r="D245" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Adjust measure range in the repeat-sign question
Extend the range from measures 1-200 to 1-220.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/msu-bench.xlsx
+++ b/msu-bench.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -5254,7 +5254,7 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>In measures 1–200, is there a repeat sign?</t>
+          <t>In measures 1–220, is there a repeat sign?</t>
         </is>
       </c>
       <c r="D245" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Generalise a playing-technique question
Replace the painting-specific phrasing with a question about the piece
and update the answer to the techniques actually present in the score.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/msu-bench.xlsx
+++ b/msu-bench.xlsx
@@ -24855,12 +24855,12 @@
       </c>
       <c r="C1225" s="3" t="inlineStr">
         <is>
-          <t>What playing techniques can be used to showcase the characteristics of different paintings?</t>
+          <t>What playing techniques are used in the piece?</t>
         </is>
       </c>
       <c r="D1225" s="5" t="inlineStr">
         <is>
-          <t>Arpeggiatio; Staccato; Tremolo Pedaling; Soft Pedal</t>
+          <t>Slur; Staccato; Tenuto; Tremolo; Marcato; Accent; Soft pedal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Break down playing techniques per painting
Restore the painting-specific question and list the techniques for each
of the ten pictures instead of a single flat set.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/msu-bench.xlsx
+++ b/msu-bench.xlsx
@@ -24855,12 +24855,12 @@
       </c>
       <c r="C1225" s="3" t="inlineStr">
         <is>
-          <t>What playing techniques are used in the piece?</t>
+          <t>What playing techniques are used to showcase the characteristics of each painting?</t>
         </is>
       </c>
       <c r="D1225" s="5" t="inlineStr">
         <is>
-          <t>Slur; Staccato; Tenuto; Tremolo; Marcato; Accent; Soft pedal</t>
+          <t>Picture 1: Slur, Marcato; Picture 2: Slur, Staccato, Tenuto; Picture 3: Slur, Staccato; Picture 4: Tenuto, Slur, Staccato, Soft pedal; Picture 5: Slur, Accent, Marcato; Picture 6: Slur, Tenuto, Staccato, Marcato, Accent; Picture 7: Staccato, Slur; Picture 8: Tremolo, Slur; Picture 9: Slur, Marcato, Tremolo; Picture 10: Slur, Marcato, Tremolo</t>
         </is>
       </c>
     </row>

</xml_diff>